<commit_message>
commiting new test scripts
</commit_message>
<xml_diff>
--- a/test-data/checkout_test_data.xlsx
+++ b/test-data/checkout_test_data.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ram\PycharmProjects\Ironman-Framework\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\PycharmProjects\Ironman-Framework\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A85D6A24-D613-4A25-8D09-147176C733CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BBC5EE-B55C-4230-AD14-D9850E8E18E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CheckoutData" sheetId="1" r:id="rId1"/>
+    <sheet name="searchproduct" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="101">
   <si>
     <t>Email</t>
   </si>
@@ -311,6 +312,18 @@
   </si>
   <si>
     <t>9876543219</t>
+  </si>
+  <si>
+    <t>searchproduct</t>
+  </si>
+  <si>
+    <t>fish food</t>
+  </si>
+  <si>
+    <t>cat food</t>
+  </si>
+  <si>
+    <t>dog food</t>
   </si>
 </sst>
 </file>
@@ -985,4 +998,37 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC082C83-A218-437C-B786-9BFED2F3383F}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>